<commit_message>
Adjusted the way some graphs looked, attempted to see if calculating female visiting nests alone was possible.
</commit_message>
<xml_diff>
--- a/UW_Nest_Behavioral_Sheets_Cleaned.xlsx
+++ b/UW_Nest_Behavioral_Sheets_Cleaned.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jacobchung/coding_projects/Owrasse_Underwater_Behavioral_Sheet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CC1BF81-6568-6046-921D-8607D8A090BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA7F80ED-1701-B745-ACEE-4BD5D5C37D0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="27760" windowHeight="17500" activeTab="1" xr2:uid="{F3336806-D2AA-0243-9E92-F92A9E05C0A5}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="27760" windowHeight="17500" xr2:uid="{F3336806-D2AA-0243-9E92-F92A9E05C0A5}"/>
   </bookViews>
   <sheets>
     <sheet name="UW_Behavior_Sheets" sheetId="1" r:id="rId1"/>
@@ -84,7 +84,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="959" uniqueCount="348">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="965" uniqueCount="354">
   <si>
     <t>Date</t>
   </si>
@@ -3191,12 +3191,30 @@
   <si>
     <t>By Association</t>
   </si>
+  <si>
+    <t>total_female visits =</t>
+  </si>
+  <si>
+    <t>female_visits_by_nm =</t>
+  </si>
+  <si>
+    <t>female_visits_by_sat =</t>
+  </si>
+  <si>
+    <t>female_visits_by_pass =</t>
+  </si>
+  <si>
+    <t xml:space="preserve">female_visits_by_snk = </t>
+  </si>
+  <si>
+    <t>female_visits_alone =</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -3318,6 +3336,13 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="16">
     <fill>
@@ -3411,7 +3436,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="31">
+  <borders count="32">
     <border>
       <left/>
       <right/>
@@ -3835,11 +3860,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="142">
+  <cellXfs count="151">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -4048,6 +4084,27 @@
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4394,7 +4451,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA17F031-50A9-714D-81FC-E69EC4191101}">
-  <dimension ref="A1:BS143"/>
+  <dimension ref="A1:BS151"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="1"/>
@@ -34656,7 +34713,6 @@
       <c r="AF143" s="22"/>
       <c r="AG143" s="22"/>
       <c r="AH143" s="22"/>
-      <c r="AI143" s="22"/>
       <c r="AJ143" s="22"/>
       <c r="AK143" s="22"/>
       <c r="AL143" s="22"/>
@@ -34693,7 +34749,102 @@
       <c r="BQ143" s="22"/>
       <c r="BR143" s="22"/>
     </row>
+    <row r="147" spans="28:43" x14ac:dyDescent="0.2">
+      <c r="AB147" s="145" t="s">
+        <v>348</v>
+      </c>
+      <c r="AC147" s="146"/>
+      <c r="AD147" s="146"/>
+      <c r="AE147" s="147"/>
+      <c r="AF147" s="142">
+        <f>SUM(AI2:AI142)</f>
+        <v>2025</v>
+      </c>
+      <c r="AG147" s="143"/>
+      <c r="AH147" s="144"/>
+      <c r="AJ147" s="142" t="s">
+        <v>353</v>
+      </c>
+      <c r="AK147" s="143"/>
+      <c r="AL147" s="143"/>
+      <c r="AM147" s="144"/>
+      <c r="AN147" s="142">
+        <f>2025-SUM(AF148:AH151)</f>
+        <v>0</v>
+      </c>
+      <c r="AO147" s="143"/>
+      <c r="AP147" s="143"/>
+      <c r="AQ147" s="144"/>
+    </row>
+    <row r="148" spans="28:43" x14ac:dyDescent="0.2">
+      <c r="AB148" s="145" t="s">
+        <v>349</v>
+      </c>
+      <c r="AC148" s="146"/>
+      <c r="AD148" s="146"/>
+      <c r="AE148" s="147"/>
+      <c r="AF148" s="142">
+        <f>SUM(O2:O142)</f>
+        <v>1563</v>
+      </c>
+      <c r="AG148" s="143"/>
+      <c r="AH148" s="144"/>
+    </row>
+    <row r="149" spans="28:43" x14ac:dyDescent="0.2">
+      <c r="AB149" s="142" t="s">
+        <v>350</v>
+      </c>
+      <c r="AC149" s="143"/>
+      <c r="AD149" s="143"/>
+      <c r="AE149" s="144"/>
+      <c r="AF149" s="142">
+        <f>SUM(P2:P142)</f>
+        <v>207</v>
+      </c>
+      <c r="AG149" s="143"/>
+      <c r="AH149" s="144"/>
+    </row>
+    <row r="150" spans="28:43" x14ac:dyDescent="0.2">
+      <c r="AB150" s="148" t="s">
+        <v>351</v>
+      </c>
+      <c r="AC150" s="149"/>
+      <c r="AD150" s="149"/>
+      <c r="AE150" s="150"/>
+      <c r="AF150" s="142">
+        <f>SUM(Q2:Q142)</f>
+        <v>222</v>
+      </c>
+      <c r="AG150" s="143"/>
+      <c r="AH150" s="144"/>
+    </row>
+    <row r="151" spans="28:43" x14ac:dyDescent="0.2">
+      <c r="AB151" s="142" t="s">
+        <v>352</v>
+      </c>
+      <c r="AC151" s="143"/>
+      <c r="AD151" s="143"/>
+      <c r="AE151" s="144"/>
+      <c r="AF151" s="142">
+        <f>SUM(R2:R142)</f>
+        <v>33</v>
+      </c>
+      <c r="AG151" s="143"/>
+      <c r="AH151" s="144"/>
+    </row>
   </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="AN147:AQ147"/>
+    <mergeCell ref="AB149:AE149"/>
+    <mergeCell ref="AB150:AE150"/>
+    <mergeCell ref="AB151:AE151"/>
+    <mergeCell ref="AJ147:AM147"/>
+    <mergeCell ref="AF147:AH147"/>
+    <mergeCell ref="AF148:AH148"/>
+    <mergeCell ref="AF149:AH149"/>
+    <mergeCell ref="AF150:AH150"/>
+    <mergeCell ref="AF151:AH151"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>

</xml_diff>